<commit_message>
Fix: Article duration manual overrides, robust unit detection for complex billing modes, and TypeScript build errors for Docker readiness
</commit_message>
<xml_diff>
--- a/Tarifs 2025.xlsx
+++ b/Tarifs 2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ivry94fr-my.sharepoint.com/personal/machevalier_ivry94_fr/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\ODP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0C67A12-A937-44B2-B87F-F843ABE797FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E62F273-FD0D-4753-B32C-443DF88CBF05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-8865" windowWidth="29040" windowHeight="15720" xr2:uid="{2E231690-236F-45E4-8EE0-2FA1E1746CC4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2E231690-236F-45E4-8EE0-2FA1E1746CC4}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="229">
   <si>
     <t>Type</t>
   </si>
@@ -591,13 +591,145 @@
   </si>
   <si>
     <t>2.20</t>
+  </si>
+  <si>
+    <t>TOURNAGE DE FILMS</t>
+  </si>
+  <si>
+    <t>INSTRUCTION, AUTORISATIONS</t>
+  </si>
+  <si>
+    <t>5.01</t>
+  </si>
+  <si>
+    <t>Mise en œuvre technicien</t>
+  </si>
+  <si>
+    <t>/h</t>
+  </si>
+  <si>
+    <t>Instruction, RDV sur site, contrôle</t>
+  </si>
+  <si>
+    <t>5.02</t>
+  </si>
+  <si>
+    <t>5.03</t>
+  </si>
+  <si>
+    <t>Obtention d'autorisations administratives</t>
+  </si>
+  <si>
+    <t>forfaitaire</t>
+  </si>
+  <si>
+    <t>Mise en place de signalisation verticale</t>
+  </si>
+  <si>
+    <t>/jour/lieu</t>
+  </si>
+  <si>
+    <t>5 Panneaux max</t>
+  </si>
+  <si>
+    <t>5.10</t>
+  </si>
+  <si>
+    <t>Neutralisation ou réservation de places de stationnement</t>
+  </si>
+  <si>
+    <t>/place/jour</t>
+  </si>
+  <si>
+    <t>40 unités - Si en zone payante s'ajoute le montant prévu pour l"immonilisation de place en zone payante</t>
+  </si>
+  <si>
+    <t>OCCUPATION DU DOMAINE PUBLIC</t>
+  </si>
+  <si>
+    <t>Occupation du domaine public</t>
+  </si>
+  <si>
+    <t>5.20</t>
+  </si>
+  <si>
+    <t>5.21</t>
+  </si>
+  <si>
+    <t>5.22</t>
+  </si>
+  <si>
+    <t>10 unités - Hors espaces verts</t>
+  </si>
+  <si>
+    <t>12 unités</t>
+  </si>
+  <si>
+    <t>Occupation d'un espace vert</t>
+  </si>
+  <si>
+    <t>Câbles d'élétricité pour alimentation temporaire</t>
+  </si>
+  <si>
+    <t>8 unités</t>
+  </si>
+  <si>
+    <t>EQUIPE (Comédiens + techniciens + figurants)</t>
+  </si>
+  <si>
+    <t>5.30</t>
+  </si>
+  <si>
+    <t>/jour</t>
+  </si>
+  <si>
+    <t>5.31</t>
+  </si>
+  <si>
+    <t>5.32</t>
+  </si>
+  <si>
+    <t>5.33</t>
+  </si>
+  <si>
+    <t>5.34</t>
+  </si>
+  <si>
+    <t>5.35</t>
+  </si>
+  <si>
+    <t>Equipe réduite à 10 personnes et moins</t>
+  </si>
+  <si>
+    <t>Equipe comprenant entre 11 et 20 personnes</t>
+  </si>
+  <si>
+    <t>Equipe comprenant entre 21 et 30 personnes</t>
+  </si>
+  <si>
+    <t>Equipe comprenant entre 31 et 80 personnes</t>
+  </si>
+  <si>
+    <t>Equipe comprenant entre 81 et 150 personnes</t>
+  </si>
+  <si>
+    <t>5.36</t>
+  </si>
+  <si>
+    <t>Supplément en cas de tournage entre 20h et 8h</t>
+  </si>
+  <si>
+    <t>/nuit</t>
+  </si>
+  <si>
+    <t>OCCUPATION DE SURVOL DE LA VOIE PUBLIQUE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -609,6 +741,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -981,10 +1119,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C092CBE-94A0-4102-8A3A-F6132871AF5F}">
   <sheetPr codeName="Feuil1"/>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="1" max="1" width="50.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.33203125" customWidth="1"/>
     <col min="3" max="3" width="27.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.88671875" style="2" bestFit="1" customWidth="1"/>
@@ -1074,7 +1212,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -1100,7 +1238,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -1126,7 +1264,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
@@ -1152,7 +1290,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
@@ -1178,7 +1316,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -1204,7 +1342,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
@@ -1230,7 +1368,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="B10" t="s">
         <v>28</v>
@@ -1256,7 +1394,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="B11" t="s">
         <v>28</v>
@@ -1282,7 +1420,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="B12" t="s">
         <v>28</v>
@@ -1308,7 +1446,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="B13" t="s">
         <v>28</v>
@@ -1334,7 +1472,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="B14" t="s">
         <v>28</v>
@@ -2310,7 +2448,306 @@
         <v>133</v>
       </c>
     </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>185</v>
+      </c>
+      <c r="B53" t="s">
+        <v>186</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="E53" t="s">
+        <v>188</v>
+      </c>
+      <c r="F53" t="s">
+        <v>189</v>
+      </c>
+      <c r="G53">
+        <v>33.299999999999997</v>
+      </c>
+      <c r="H53" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>185</v>
+      </c>
+      <c r="B54" t="s">
+        <v>186</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E54" t="s">
+        <v>193</v>
+      </c>
+      <c r="F54" t="s">
+        <v>194</v>
+      </c>
+      <c r="G54">
+        <v>130.30000000000001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>185</v>
+      </c>
+      <c r="B55" t="s">
+        <v>186</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="E55" t="s">
+        <v>195</v>
+      </c>
+      <c r="F55" t="s">
+        <v>196</v>
+      </c>
+      <c r="G55">
+        <v>58.85</v>
+      </c>
+      <c r="H55" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>185</v>
+      </c>
+      <c r="B56" t="s">
+        <v>108</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="E56" t="s">
+        <v>199</v>
+      </c>
+      <c r="F56" t="s">
+        <v>200</v>
+      </c>
+      <c r="G56">
+        <v>13.1</v>
+      </c>
+      <c r="H56" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>185</v>
+      </c>
+      <c r="B57" t="s">
+        <v>202</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="E57" t="s">
+        <v>203</v>
+      </c>
+      <c r="F57" t="s">
+        <v>95</v>
+      </c>
+      <c r="G57">
+        <v>3.3</v>
+      </c>
+      <c r="H57" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>185</v>
+      </c>
+      <c r="B58" t="s">
+        <v>202</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="E58" t="s">
+        <v>209</v>
+      </c>
+      <c r="F58" t="s">
+        <v>95</v>
+      </c>
+      <c r="G58">
+        <v>3.95</v>
+      </c>
+      <c r="H58" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>185</v>
+      </c>
+      <c r="B59" t="s">
+        <v>202</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E59" t="s">
+        <v>210</v>
+      </c>
+      <c r="F59" t="s">
+        <v>72</v>
+      </c>
+      <c r="G59">
+        <v>5.25</v>
+      </c>
+      <c r="H59" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>185</v>
+      </c>
+      <c r="B60" t="s">
+        <v>212</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E60" t="s">
+        <v>220</v>
+      </c>
+      <c r="F60" t="s">
+        <v>214</v>
+      </c>
+      <c r="G60">
+        <v>326.89999999999998</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>185</v>
+      </c>
+      <c r="B61" t="s">
+        <v>212</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E61" t="s">
+        <v>221</v>
+      </c>
+      <c r="F61" t="s">
+        <v>214</v>
+      </c>
+      <c r="G61">
+        <v>653.65</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>185</v>
+      </c>
+      <c r="B62" t="s">
+        <v>212</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="E62" t="s">
+        <v>222</v>
+      </c>
+      <c r="F62" t="s">
+        <v>214</v>
+      </c>
+      <c r="G62">
+        <v>832.2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>185</v>
+      </c>
+      <c r="B63" t="s">
+        <v>212</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="E63" t="s">
+        <v>223</v>
+      </c>
+      <c r="F63" t="s">
+        <v>214</v>
+      </c>
+      <c r="G63">
+        <v>1009.6</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>185</v>
+      </c>
+      <c r="B64" t="s">
+        <v>212</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="E64" t="s">
+        <v>224</v>
+      </c>
+      <c r="F64" t="s">
+        <v>214</v>
+      </c>
+      <c r="G64">
+        <v>1199.2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>185</v>
+      </c>
+      <c r="B65" t="s">
+        <v>212</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="E65" t="s">
+        <v>220</v>
+      </c>
+      <c r="F65" t="s">
+        <v>214</v>
+      </c>
+      <c r="G65">
+        <v>331.9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>185</v>
+      </c>
+      <c r="B66" t="s">
+        <v>212</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="E66" t="s">
+        <v>226</v>
+      </c>
+      <c r="F66" t="s">
+        <v>227</v>
+      </c>
+      <c r="G66">
+        <v>416.1</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete modernization of settings, backlog and governance system
</commit_message>
<xml_diff>
--- a/Tarifs 2025.xlsx
+++ b/Tarifs 2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\ODP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E62F273-FD0D-4753-B32C-443DF88CBF05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58508624-3E1F-4F0E-AA22-14A7ADD19571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2E231690-236F-45E4-8EE0-2FA1E1746CC4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="228">
   <si>
     <t>Type</t>
   </si>
@@ -62,9 +62,6 @@
     <t>Observations</t>
   </si>
   <si>
-    <t>OCCUPATIO DE SURVOL DE LA VOIE PUBLIQUE</t>
-  </si>
-  <si>
     <t>ENSEIGNES</t>
   </si>
   <si>
@@ -626,9 +623,6 @@
     <t>Mise en place de signalisation verticale</t>
   </si>
   <si>
-    <t>/jour/lieu</t>
-  </si>
-  <si>
     <t>5 Panneaux max</t>
   </si>
   <si>
@@ -723,6 +717,9 @@
   </si>
   <si>
     <t>OCCUPATION DE SURVOL DE LA VOIE PUBLIQUE</t>
+  </si>
+  <si>
+    <t>/lieu/jour</t>
   </si>
 </sst>
 </file>
@@ -1160,334 +1157,334 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
       </c>
       <c r="G2">
         <v>19.68</v>
       </c>
       <c r="H2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>226</v>
+      </c>
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G3">
         <v>39.36</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G4">
         <v>29.52</v>
       </c>
       <c r="H4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G5">
         <v>59.04</v>
       </c>
       <c r="H5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E6" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="E6" t="s">
-        <v>20</v>
-      </c>
       <c r="F6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G6">
         <v>39.36</v>
       </c>
       <c r="H6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G7">
         <v>65.599999999999994</v>
       </c>
       <c r="H7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G8">
         <v>59.04</v>
       </c>
       <c r="H8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G9">
         <v>78.72</v>
       </c>
       <c r="H9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E10" t="s">
         <v>28</v>
       </c>
-      <c r="C10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="E10" t="s">
-        <v>29</v>
-      </c>
       <c r="F10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G10">
         <v>6.56</v>
       </c>
       <c r="H10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G11">
         <v>2.62</v>
       </c>
       <c r="H11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" t="s">
         <v>33</v>
-      </c>
-      <c r="F12" t="s">
-        <v>34</v>
       </c>
       <c r="G12">
         <v>1.31</v>
       </c>
       <c r="H12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G13">
         <v>14.43</v>
       </c>
       <c r="H13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E14" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" t="s">
         <v>38</v>
-      </c>
-      <c r="F14" t="s">
-        <v>39</v>
       </c>
       <c r="G14">
         <v>19.68</v>
@@ -1495,48 +1492,48 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s">
         <v>40</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>41</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E15" t="s">
         <v>42</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="E15" t="s">
-        <v>43</v>
-      </c>
       <c r="F15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G15">
         <v>78.72</v>
       </c>
       <c r="H15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" t="s">
         <v>40</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>41</v>
       </c>
-      <c r="C16" t="s">
-        <v>42</v>
-      </c>
       <c r="D16" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G16">
         <v>59.04</v>
@@ -1544,22 +1541,22 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" t="s">
         <v>40</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>41</v>
       </c>
-      <c r="C17" t="s">
-        <v>42</v>
-      </c>
       <c r="D17" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G17">
         <v>29.52</v>
@@ -1567,100 +1564,100 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" t="s">
         <v>40</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>41</v>
       </c>
-      <c r="C18" t="s">
-        <v>42</v>
-      </c>
       <c r="D18" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G18">
         <v>36.74</v>
       </c>
       <c r="H18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" t="s">
         <v>40</v>
       </c>
-      <c r="B19" t="s">
-        <v>41</v>
-      </c>
       <c r="C19" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E19" t="s">
         <v>49</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="E19" t="s">
-        <v>50</v>
-      </c>
       <c r="F19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G19">
         <v>23.62</v>
       </c>
       <c r="H19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" t="s">
         <v>40</v>
       </c>
-      <c r="B20" t="s">
-        <v>41</v>
-      </c>
       <c r="C20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G20">
         <v>23.62</v>
       </c>
       <c r="H20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" t="s">
         <v>40</v>
       </c>
-      <c r="B21" t="s">
-        <v>41</v>
-      </c>
       <c r="C21" t="s">
+        <v>53</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E21" t="s">
         <v>54</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="E21" t="s">
-        <v>55</v>
-      </c>
       <c r="F21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G21">
         <v>13.12</v>
@@ -1668,74 +1665,74 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" t="s">
         <v>40</v>
       </c>
-      <c r="B22" t="s">
-        <v>41</v>
-      </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G22">
         <v>62.32</v>
       </c>
       <c r="H22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>39</v>
+      </c>
+      <c r="B23" t="s">
         <v>40</v>
       </c>
-      <c r="B23" t="s">
-        <v>41</v>
-      </c>
       <c r="C23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F23" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G23">
         <v>15.74</v>
       </c>
       <c r="H23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B24" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" t="s">
         <v>60</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E24" t="s">
         <v>61</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="E24" t="s">
-        <v>62</v>
-      </c>
       <c r="F24" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G24">
         <v>62.32</v>
@@ -1743,74 +1740,74 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B25" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" t="s">
         <v>60</v>
       </c>
-      <c r="C25" t="s">
-        <v>61</v>
-      </c>
       <c r="D25" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E25" t="s">
+        <v>62</v>
+      </c>
+      <c r="F25" t="s">
         <v>63</v>
-      </c>
-      <c r="F25" t="s">
-        <v>64</v>
       </c>
       <c r="G25">
         <v>78.72</v>
       </c>
       <c r="H25" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>65</v>
+      </c>
+      <c r="B26" t="s">
         <v>66</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>67</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E26" t="s">
         <v>68</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="E26" t="s">
-        <v>69</v>
-      </c>
       <c r="F26" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G26">
         <v>16.399999999999999</v>
       </c>
       <c r="H26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
+        <v>65</v>
+      </c>
+      <c r="B27" t="s">
         <v>66</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>67</v>
       </c>
-      <c r="C27" t="s">
-        <v>68</v>
-      </c>
       <c r="D27" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E27" t="s">
+        <v>70</v>
+      </c>
+      <c r="F27" t="s">
         <v>71</v>
-      </c>
-      <c r="F27" t="s">
-        <v>72</v>
       </c>
       <c r="G27">
         <v>65.599999999999994</v>
@@ -1818,22 +1815,22 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>65</v>
+      </c>
+      <c r="B28" t="s">
         <v>66</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>67</v>
       </c>
-      <c r="C28" t="s">
-        <v>68</v>
-      </c>
       <c r="D28" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F28" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G28">
         <v>7.87</v>
@@ -1841,152 +1838,152 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" t="s">
         <v>66</v>
       </c>
-      <c r="B29" t="s">
-        <v>67</v>
-      </c>
       <c r="C29" t="s">
+        <v>73</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E29" t="s">
         <v>74</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
         <v>75</v>
-      </c>
-      <c r="F29" t="s">
-        <v>76</v>
       </c>
       <c r="G29">
         <v>22.96</v>
       </c>
       <c r="H29" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>65</v>
+      </c>
+      <c r="B30" t="s">
         <v>66</v>
       </c>
-      <c r="B30" t="s">
-        <v>67</v>
-      </c>
       <c r="C30" t="s">
+        <v>77</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E30" t="s">
         <v>78</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="E30" t="s">
-        <v>79</v>
-      </c>
       <c r="F30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G30">
         <v>13.12</v>
       </c>
       <c r="H30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>65</v>
+      </c>
+      <c r="B31" t="s">
         <v>66</v>
       </c>
-      <c r="B31" t="s">
-        <v>67</v>
-      </c>
       <c r="C31" t="s">
+        <v>79</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E31" t="s">
         <v>80</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="E31" t="s">
-        <v>81</v>
-      </c>
       <c r="F31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G31">
         <v>3.94</v>
       </c>
       <c r="H31" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>65</v>
+      </c>
+      <c r="B32" t="s">
         <v>66</v>
       </c>
-      <c r="B32" t="s">
-        <v>67</v>
-      </c>
       <c r="C32" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E32" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F32" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G32">
         <v>6.56</v>
       </c>
       <c r="H32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>65</v>
+      </c>
+      <c r="B33" t="s">
         <v>66</v>
       </c>
-      <c r="B33" t="s">
-        <v>67</v>
-      </c>
       <c r="C33" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E33" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F33" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G33">
         <v>13.12</v>
       </c>
       <c r="H33" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>65</v>
+      </c>
+      <c r="B34" t="s">
         <v>66</v>
       </c>
-      <c r="B34" t="s">
-        <v>67</v>
-      </c>
       <c r="C34" t="s">
+        <v>86</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E34" t="s">
         <v>87</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="E34" t="s">
-        <v>88</v>
-      </c>
       <c r="F34" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G34">
         <v>5.25</v>
@@ -1994,22 +1991,22 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>65</v>
+      </c>
+      <c r="B35" t="s">
         <v>66</v>
       </c>
-      <c r="B35" t="s">
-        <v>67</v>
-      </c>
       <c r="C35" t="s">
+        <v>88</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E35" t="s">
         <v>89</v>
       </c>
-      <c r="D35" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
         <v>90</v>
-      </c>
-      <c r="F35" t="s">
-        <v>91</v>
       </c>
       <c r="G35">
         <v>295.2</v>
@@ -2017,48 +2014,48 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B36" t="s">
+        <v>91</v>
+      </c>
+      <c r="C36" t="s">
         <v>92</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E36" t="s">
         <v>93</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E36" t="s">
+      <c r="F36" t="s">
         <v>94</v>
-      </c>
-      <c r="F36" t="s">
-        <v>95</v>
       </c>
       <c r="G36">
         <v>1.31</v>
       </c>
       <c r="H36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B37" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37" t="s">
         <v>92</v>
       </c>
-      <c r="C37" t="s">
-        <v>93</v>
-      </c>
       <c r="D37" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E37" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F37" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G37">
         <v>6.56</v>
@@ -2066,126 +2063,126 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B38" t="s">
+        <v>91</v>
+      </c>
+      <c r="C38" t="s">
         <v>92</v>
       </c>
-      <c r="C38" t="s">
-        <v>93</v>
-      </c>
       <c r="D38" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E38" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F38" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G38">
         <v>164</v>
       </c>
       <c r="H38" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B39" t="s">
+        <v>91</v>
+      </c>
+      <c r="C39" t="s">
         <v>92</v>
       </c>
-      <c r="C39" t="s">
-        <v>93</v>
-      </c>
       <c r="D39" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E39" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F39" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G39">
         <v>13.12</v>
       </c>
       <c r="H39" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B40" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C40" t="s">
+        <v>101</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="E40" t="s">
         <v>102</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
         <v>103</v>
-      </c>
-      <c r="F40" t="s">
-        <v>104</v>
       </c>
       <c r="G40">
         <v>8.1999999999999993</v>
       </c>
       <c r="H40" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B41" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C41" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E41" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F41" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G41">
         <v>9.84</v>
       </c>
       <c r="H41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B42" t="s">
+        <v>107</v>
+      </c>
+      <c r="C42" t="s">
+        <v>60</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="E42" t="s">
         <v>108</v>
       </c>
-      <c r="C42" t="s">
-        <v>61</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E42" t="s">
-        <v>109</v>
-      </c>
       <c r="F42" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G42">
         <v>3.94</v>
@@ -2193,100 +2190,100 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C43" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E43" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F43" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G43">
         <v>13.12</v>
       </c>
       <c r="H43" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B44" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C44" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E44" t="s">
+        <v>111</v>
+      </c>
+      <c r="F44" t="s">
         <v>112</v>
-      </c>
-      <c r="F44" t="s">
-        <v>113</v>
       </c>
       <c r="G44">
         <v>869.2</v>
       </c>
       <c r="H44" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B45" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C45" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E45" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F45" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G45">
         <v>901.34</v>
       </c>
       <c r="H45" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B46" t="s">
+        <v>115</v>
+      </c>
+      <c r="C46" t="s">
         <v>116</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E46" t="s">
         <v>117</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="E46" t="s">
-        <v>118</v>
-      </c>
       <c r="F46" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G46">
         <v>3.28</v>
@@ -2294,198 +2291,198 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B47" t="s">
+        <v>115</v>
+      </c>
+      <c r="C47" t="s">
         <v>116</v>
       </c>
-      <c r="C47" t="s">
-        <v>117</v>
-      </c>
       <c r="D47" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E47" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F47" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G47">
         <v>3.94</v>
       </c>
       <c r="H47" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B48" t="s">
+        <v>115</v>
+      </c>
+      <c r="C48" t="s">
         <v>116</v>
       </c>
-      <c r="C48" t="s">
-        <v>117</v>
-      </c>
       <c r="D48" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E48" t="s">
+        <v>119</v>
+      </c>
+      <c r="F48" t="s">
         <v>120</v>
-      </c>
-      <c r="F48" t="s">
-        <v>121</v>
       </c>
       <c r="G48">
         <v>62.98</v>
       </c>
       <c r="H48" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B49" t="s">
+        <v>115</v>
+      </c>
+      <c r="C49" t="s">
         <v>116</v>
       </c>
-      <c r="C49" t="s">
-        <v>117</v>
-      </c>
       <c r="D49" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E49" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G49">
         <v>0</v>
       </c>
       <c r="H49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B50" t="s">
+        <v>115</v>
+      </c>
+      <c r="C50" t="s">
         <v>116</v>
       </c>
-      <c r="C50" t="s">
-        <v>117</v>
-      </c>
       <c r="D50" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E50" t="s">
+        <v>124</v>
+      </c>
+      <c r="F50" t="s">
         <v>125</v>
-      </c>
-      <c r="F50" t="s">
-        <v>126</v>
       </c>
       <c r="G50">
         <v>11.48</v>
       </c>
       <c r="H50" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B51" t="s">
+        <v>115</v>
+      </c>
+      <c r="C51" t="s">
         <v>116</v>
       </c>
-      <c r="C51" t="s">
-        <v>117</v>
-      </c>
       <c r="D51" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E51" t="s">
+        <v>127</v>
+      </c>
+      <c r="F51" t="s">
         <v>128</v>
-      </c>
-      <c r="F51" t="s">
-        <v>129</v>
       </c>
       <c r="G51">
         <v>0.98</v>
       </c>
       <c r="H51" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B52" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C52" t="s">
+        <v>130</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E52" t="s">
         <v>131</v>
       </c>
-      <c r="D52" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="E52" t="s">
-        <v>132</v>
-      </c>
       <c r="F52" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G52">
         <v>80.69</v>
       </c>
       <c r="H52" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
+        <v>184</v>
+      </c>
+      <c r="B53" t="s">
         <v>185</v>
       </c>
-      <c r="B53" t="s">
+      <c r="D53" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="D53" s="2" t="s">
+      <c r="E53" t="s">
         <v>187</v>
       </c>
-      <c r="E53" t="s">
+      <c r="F53" t="s">
         <v>188</v>
-      </c>
-      <c r="F53" t="s">
-        <v>189</v>
       </c>
       <c r="G53">
         <v>33.299999999999997</v>
       </c>
       <c r="H53" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
+        <v>184</v>
+      </c>
+      <c r="B54" t="s">
         <v>185</v>
       </c>
-      <c r="B54" t="s">
-        <v>186</v>
-      </c>
       <c r="D54" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E54" t="s">
+        <v>192</v>
+      </c>
+      <c r="F54" t="s">
         <v>193</v>
-      </c>
-      <c r="F54" t="s">
-        <v>194</v>
       </c>
       <c r="G54">
         <v>130.30000000000001</v>
@@ -2493,134 +2490,134 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
+        <v>184</v>
+      </c>
+      <c r="B55" t="s">
         <v>185</v>
       </c>
-      <c r="B55" t="s">
-        <v>186</v>
-      </c>
       <c r="D55" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E55" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F55" t="s">
-        <v>196</v>
+        <v>227</v>
       </c>
       <c r="G55">
         <v>58.85</v>
       </c>
       <c r="H55" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B56" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D56" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E56" t="s">
+        <v>197</v>
+      </c>
+      <c r="F56" t="s">
         <v>198</v>
-      </c>
-      <c r="E56" t="s">
-        <v>199</v>
-      </c>
-      <c r="F56" t="s">
-        <v>200</v>
       </c>
       <c r="G56">
         <v>13.1</v>
       </c>
       <c r="H56" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B57" t="s">
+        <v>200</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="D57" s="2" t="s">
-        <v>204</v>
-      </c>
       <c r="E57" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F57" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G57">
         <v>3.3</v>
       </c>
       <c r="H57" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B58" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="E58" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F58" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G58">
         <v>3.95</v>
       </c>
       <c r="H58" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B59" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E59" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F59" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G59">
         <v>5.25</v>
       </c>
       <c r="H59" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B60" t="s">
+        <v>210</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E60" t="s">
+        <v>218</v>
+      </c>
+      <c r="F60" t="s">
         <v>212</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="E60" t="s">
-        <v>220</v>
-      </c>
-      <c r="F60" t="s">
-        <v>214</v>
       </c>
       <c r="G60">
         <v>326.89999999999998</v>
@@ -2628,19 +2625,19 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B61" t="s">
+        <v>210</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E61" t="s">
+        <v>219</v>
+      </c>
+      <c r="F61" t="s">
         <v>212</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="E61" t="s">
-        <v>221</v>
-      </c>
-      <c r="F61" t="s">
-        <v>214</v>
       </c>
       <c r="G61">
         <v>653.65</v>
@@ -2648,19 +2645,19 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B62" t="s">
+        <v>210</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="E62" t="s">
+        <v>220</v>
+      </c>
+      <c r="F62" t="s">
         <v>212</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="E62" t="s">
-        <v>222</v>
-      </c>
-      <c r="F62" t="s">
-        <v>214</v>
       </c>
       <c r="G62">
         <v>832.2</v>
@@ -2668,19 +2665,19 @@
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B63" t="s">
+        <v>210</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E63" t="s">
+        <v>221</v>
+      </c>
+      <c r="F63" t="s">
         <v>212</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="E63" t="s">
-        <v>223</v>
-      </c>
-      <c r="F63" t="s">
-        <v>214</v>
       </c>
       <c r="G63">
         <v>1009.6</v>
@@ -2688,19 +2685,19 @@
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B64" t="s">
+        <v>210</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="E64" t="s">
+        <v>222</v>
+      </c>
+      <c r="F64" t="s">
         <v>212</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="E64" t="s">
-        <v>224</v>
-      </c>
-      <c r="F64" t="s">
-        <v>214</v>
       </c>
       <c r="G64">
         <v>1199.2</v>
@@ -2708,19 +2705,19 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B65" t="s">
+        <v>210</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="E65" t="s">
+        <v>218</v>
+      </c>
+      <c r="F65" t="s">
         <v>212</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="E65" t="s">
-        <v>220</v>
-      </c>
-      <c r="F65" t="s">
-        <v>214</v>
       </c>
       <c r="G65">
         <v>331.9</v>
@@ -2728,19 +2725,19 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B66" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D66" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="E66" t="s">
+        <v>224</v>
+      </c>
+      <c r="F66" t="s">
         <v>225</v>
-      </c>
-      <c r="E66" t="s">
-        <v>226</v>
-      </c>
-      <c r="F66" t="s">
-        <v>227</v>
       </c>
       <c r="G66">
         <v>416.1</v>

</xml_diff>